<commit_message>
Prepare Vercel PostgreSQL deployment
</commit_message>
<xml_diff>
--- a/Proposta de medição/Proposta_de_medição MODELO.xlsx
+++ b/Proposta de medição/Proposta_de_medição MODELO.xlsx
@@ -264,22 +264,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t/>
+          <t>SERVIÇOS</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t/>
+          <t>BLOCO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t/>
+          <t>CASA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t/>
+          <t>OBSERVAÇÕES</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">

</xml_diff>